<commit_message>
Running from my mac
</commit_message>
<xml_diff>
--- a/models/image_results_hundred2.xlsx
+++ b/models/image_results_hundred2.xlsx
@@ -17,16 +17,13 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="1">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -37,7 +34,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -45,21 +42,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin"/>
-      <right style="thin"/>
-      <top style="thin"/>
-      <bottom style="thin"/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -429,19 +417,19 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>true index</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>predicted index</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="1" t="n">
+      <c r="A2" t="n">
         <v>0</v>
       </c>
       <c r="B2" t="n">
@@ -452,7 +440,7 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="1" t="n">
+      <c r="A3" t="n">
         <v>1</v>
       </c>
       <c r="B3" t="n">
@@ -463,7 +451,7 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="1" t="n">
+      <c r="A4" t="n">
         <v>2</v>
       </c>
       <c r="B4" t="n">
@@ -474,7 +462,7 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="1" t="n">
+      <c r="A5" t="n">
         <v>3</v>
       </c>
       <c r="B5" t="n">
@@ -485,7 +473,7 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="1" t="n">
+      <c r="A6" t="n">
         <v>4</v>
       </c>
       <c r="B6" t="n">
@@ -496,7 +484,7 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="1" t="n">
+      <c r="A7" t="n">
         <v>5</v>
       </c>
       <c r="B7" t="n">
@@ -507,7 +495,7 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="1" t="n">
+      <c r="A8" t="n">
         <v>6</v>
       </c>
       <c r="B8" t="n">
@@ -518,7 +506,7 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="1" t="n">
+      <c r="A9" t="n">
         <v>7</v>
       </c>
       <c r="B9" t="n">
@@ -529,7 +517,7 @@
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="1" t="n">
+      <c r="A10" t="n">
         <v>8</v>
       </c>
       <c r="B10" t="n">
@@ -540,7 +528,7 @@
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="1" t="n">
+      <c r="A11" t="n">
         <v>9</v>
       </c>
       <c r="B11" t="n">
@@ -551,7 +539,7 @@
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="1" t="n">
+      <c r="A12" t="n">
         <v>10</v>
       </c>
       <c r="B12" t="n">
@@ -562,7 +550,7 @@
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="1" t="n">
+      <c r="A13" t="n">
         <v>11</v>
       </c>
       <c r="B13" t="n">
@@ -573,7 +561,7 @@
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="1" t="n">
+      <c r="A14" t="n">
         <v>12</v>
       </c>
       <c r="B14" t="n">
@@ -584,7 +572,7 @@
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="1" t="n">
+      <c r="A15" t="n">
         <v>13</v>
       </c>
       <c r="B15" t="n">
@@ -595,7 +583,7 @@
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="1" t="n">
+      <c r="A16" t="n">
         <v>14</v>
       </c>
       <c r="B16" t="n">
@@ -606,7 +594,7 @@
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="1" t="n">
+      <c r="A17" t="n">
         <v>15</v>
       </c>
       <c r="B17" t="n">
@@ -617,7 +605,7 @@
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="1" t="n">
+      <c r="A18" t="n">
         <v>16</v>
       </c>
       <c r="B18" t="n">
@@ -628,7 +616,7 @@
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="1" t="n">
+      <c r="A19" t="n">
         <v>17</v>
       </c>
       <c r="B19" t="n">
@@ -639,7 +627,7 @@
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="1" t="n">
+      <c r="A20" t="n">
         <v>18</v>
       </c>
       <c r="B20" t="n">
@@ -650,7 +638,7 @@
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="1" t="n">
+      <c r="A21" t="n">
         <v>19</v>
       </c>
       <c r="B21" t="n">
@@ -661,7 +649,7 @@
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="1" t="n">
+      <c r="A22" t="n">
         <v>20</v>
       </c>
       <c r="B22" t="n">
@@ -672,7 +660,7 @@
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="1" t="n">
+      <c r="A23" t="n">
         <v>21</v>
       </c>
       <c r="B23" t="n">
@@ -683,7 +671,7 @@
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="1" t="n">
+      <c r="A24" t="n">
         <v>22</v>
       </c>
       <c r="B24" t="n">
@@ -694,7 +682,7 @@
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="1" t="n">
+      <c r="A25" t="n">
         <v>23</v>
       </c>
       <c r="B25" t="n">
@@ -705,7 +693,7 @@
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="1" t="n">
+      <c r="A26" t="n">
         <v>24</v>
       </c>
       <c r="B26" t="n">
@@ -716,7 +704,7 @@
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="1" t="n">
+      <c r="A27" t="n">
         <v>25</v>
       </c>
       <c r="B27" t="n">
@@ -727,7 +715,7 @@
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="1" t="n">
+      <c r="A28" t="n">
         <v>26</v>
       </c>
       <c r="B28" t="n">
@@ -738,7 +726,7 @@
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="1" t="n">
+      <c r="A29" t="n">
         <v>27</v>
       </c>
       <c r="B29" t="n">
@@ -749,7 +737,7 @@
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="1" t="n">
+      <c r="A30" t="n">
         <v>28</v>
       </c>
       <c r="B30" t="n">
@@ -760,7 +748,7 @@
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="1" t="n">
+      <c r="A31" t="n">
         <v>29</v>
       </c>
       <c r="B31" t="n">
@@ -771,7 +759,7 @@
       </c>
     </row>
     <row r="32">
-      <c r="A32" s="1" t="n">
+      <c r="A32" t="n">
         <v>30</v>
       </c>
       <c r="B32" t="n">
@@ -782,7 +770,7 @@
       </c>
     </row>
     <row r="33">
-      <c r="A33" s="1" t="n">
+      <c r="A33" t="n">
         <v>31</v>
       </c>
       <c r="B33" t="n">
@@ -793,7 +781,7 @@
       </c>
     </row>
     <row r="34">
-      <c r="A34" s="1" t="n">
+      <c r="A34" t="n">
         <v>32</v>
       </c>
       <c r="B34" t="n">
@@ -804,7 +792,7 @@
       </c>
     </row>
     <row r="35">
-      <c r="A35" s="1" t="n">
+      <c r="A35" t="n">
         <v>33</v>
       </c>
       <c r="B35" t="n">
@@ -815,7 +803,7 @@
       </c>
     </row>
     <row r="36">
-      <c r="A36" s="1" t="n">
+      <c r="A36" t="n">
         <v>34</v>
       </c>
       <c r="B36" t="n">
@@ -826,7 +814,7 @@
       </c>
     </row>
     <row r="37">
-      <c r="A37" s="1" t="n">
+      <c r="A37" t="n">
         <v>35</v>
       </c>
       <c r="B37" t="n">
@@ -837,7 +825,7 @@
       </c>
     </row>
     <row r="38">
-      <c r="A38" s="1" t="n">
+      <c r="A38" t="n">
         <v>36</v>
       </c>
       <c r="B38" t="n">
@@ -848,7 +836,7 @@
       </c>
     </row>
     <row r="39">
-      <c r="A39" s="1" t="n">
+      <c r="A39" t="n">
         <v>37</v>
       </c>
       <c r="B39" t="n">
@@ -859,7 +847,7 @@
       </c>
     </row>
     <row r="40">
-      <c r="A40" s="1" t="n">
+      <c r="A40" t="n">
         <v>38</v>
       </c>
       <c r="B40" t="n">
@@ -870,7 +858,7 @@
       </c>
     </row>
     <row r="41">
-      <c r="A41" s="1" t="n">
+      <c r="A41" t="n">
         <v>39</v>
       </c>
       <c r="B41" t="n">
@@ -881,7 +869,7 @@
       </c>
     </row>
     <row r="42">
-      <c r="A42" s="1" t="n">
+      <c r="A42" t="n">
         <v>40</v>
       </c>
       <c r="B42" t="n">
@@ -892,7 +880,7 @@
       </c>
     </row>
     <row r="43">
-      <c r="A43" s="1" t="n">
+      <c r="A43" t="n">
         <v>41</v>
       </c>
       <c r="B43" t="n">
@@ -903,7 +891,7 @@
       </c>
     </row>
     <row r="44">
-      <c r="A44" s="1" t="n">
+      <c r="A44" t="n">
         <v>42</v>
       </c>
       <c r="B44" t="n">
@@ -914,7 +902,7 @@
       </c>
     </row>
     <row r="45">
-      <c r="A45" s="1" t="n">
+      <c r="A45" t="n">
         <v>43</v>
       </c>
       <c r="B45" t="n">
@@ -925,7 +913,7 @@
       </c>
     </row>
     <row r="46">
-      <c r="A46" s="1" t="n">
+      <c r="A46" t="n">
         <v>44</v>
       </c>
       <c r="B46" t="n">
@@ -936,7 +924,7 @@
       </c>
     </row>
     <row r="47">
-      <c r="A47" s="1" t="n">
+      <c r="A47" t="n">
         <v>45</v>
       </c>
       <c r="B47" t="n">
@@ -947,7 +935,7 @@
       </c>
     </row>
     <row r="48">
-      <c r="A48" s="1" t="n">
+      <c r="A48" t="n">
         <v>46</v>
       </c>
       <c r="B48" t="n">
@@ -958,7 +946,7 @@
       </c>
     </row>
     <row r="49">
-      <c r="A49" s="1" t="n">
+      <c r="A49" t="n">
         <v>47</v>
       </c>
       <c r="B49" t="n">
@@ -969,7 +957,7 @@
       </c>
     </row>
     <row r="50">
-      <c r="A50" s="1" t="n">
+      <c r="A50" t="n">
         <v>48</v>
       </c>
       <c r="B50" t="n">
@@ -980,7 +968,7 @@
       </c>
     </row>
     <row r="51">
-      <c r="A51" s="1" t="n">
+      <c r="A51" t="n">
         <v>49</v>
       </c>
       <c r="B51" t="n">
@@ -991,7 +979,7 @@
       </c>
     </row>
     <row r="52">
-      <c r="A52" s="1" t="n">
+      <c r="A52" t="n">
         <v>50</v>
       </c>
       <c r="B52" t="n">
@@ -1002,7 +990,7 @@
       </c>
     </row>
     <row r="53">
-      <c r="A53" s="1" t="n">
+      <c r="A53" t="n">
         <v>51</v>
       </c>
       <c r="B53" t="n">
@@ -1013,7 +1001,7 @@
       </c>
     </row>
     <row r="54">
-      <c r="A54" s="1" t="n">
+      <c r="A54" t="n">
         <v>52</v>
       </c>
       <c r="B54" t="n">
@@ -1024,7 +1012,7 @@
       </c>
     </row>
     <row r="55">
-      <c r="A55" s="1" t="n">
+      <c r="A55" t="n">
         <v>53</v>
       </c>
       <c r="B55" t="n">
@@ -1035,7 +1023,7 @@
       </c>
     </row>
     <row r="56">
-      <c r="A56" s="1" t="n">
+      <c r="A56" t="n">
         <v>54</v>
       </c>
       <c r="B56" t="n">
@@ -1046,7 +1034,7 @@
       </c>
     </row>
     <row r="57">
-      <c r="A57" s="1" t="n">
+      <c r="A57" t="n">
         <v>55</v>
       </c>
       <c r="B57" t="n">
@@ -1057,7 +1045,7 @@
       </c>
     </row>
     <row r="58">
-      <c r="A58" s="1" t="n">
+      <c r="A58" t="n">
         <v>56</v>
       </c>
       <c r="B58" t="n">
@@ -1068,7 +1056,7 @@
       </c>
     </row>
     <row r="59">
-      <c r="A59" s="1" t="n">
+      <c r="A59" t="n">
         <v>57</v>
       </c>
       <c r="B59" t="n">
@@ -1079,7 +1067,7 @@
       </c>
     </row>
     <row r="60">
-      <c r="A60" s="1" t="n">
+      <c r="A60" t="n">
         <v>58</v>
       </c>
       <c r="B60" t="n">
@@ -1090,7 +1078,7 @@
       </c>
     </row>
     <row r="61">
-      <c r="A61" s="1" t="n">
+      <c r="A61" t="n">
         <v>59</v>
       </c>
       <c r="B61" t="n">
@@ -1101,7 +1089,7 @@
       </c>
     </row>
     <row r="62">
-      <c r="A62" s="1" t="n">
+      <c r="A62" t="n">
         <v>60</v>
       </c>
       <c r="B62" t="n">
@@ -1112,7 +1100,7 @@
       </c>
     </row>
     <row r="63">
-      <c r="A63" s="1" t="n">
+      <c r="A63" t="n">
         <v>61</v>
       </c>
       <c r="B63" t="n">
@@ -1123,7 +1111,7 @@
       </c>
     </row>
     <row r="64">
-      <c r="A64" s="1" t="n">
+      <c r="A64" t="n">
         <v>62</v>
       </c>
       <c r="B64" t="n">
@@ -1134,7 +1122,7 @@
       </c>
     </row>
     <row r="65">
-      <c r="A65" s="1" t="n">
+      <c r="A65" t="n">
         <v>63</v>
       </c>
       <c r="B65" t="n">
@@ -1145,7 +1133,7 @@
       </c>
     </row>
     <row r="66">
-      <c r="A66" s="1" t="n">
+      <c r="A66" t="n">
         <v>64</v>
       </c>
       <c r="B66" t="n">
@@ -1156,7 +1144,7 @@
       </c>
     </row>
     <row r="67">
-      <c r="A67" s="1" t="n">
+      <c r="A67" t="n">
         <v>65</v>
       </c>
       <c r="B67" t="n">
@@ -1167,7 +1155,7 @@
       </c>
     </row>
     <row r="68">
-      <c r="A68" s="1" t="n">
+      <c r="A68" t="n">
         <v>66</v>
       </c>
       <c r="B68" t="n">
@@ -1178,7 +1166,7 @@
       </c>
     </row>
     <row r="69">
-      <c r="A69" s="1" t="n">
+      <c r="A69" t="n">
         <v>67</v>
       </c>
       <c r="B69" t="n">
@@ -1189,7 +1177,7 @@
       </c>
     </row>
     <row r="70">
-      <c r="A70" s="1" t="n">
+      <c r="A70" t="n">
         <v>68</v>
       </c>
       <c r="B70" t="n">
@@ -1200,7 +1188,7 @@
       </c>
     </row>
     <row r="71">
-      <c r="A71" s="1" t="n">
+      <c r="A71" t="n">
         <v>69</v>
       </c>
       <c r="B71" t="n">
@@ -1211,7 +1199,7 @@
       </c>
     </row>
     <row r="72">
-      <c r="A72" s="1" t="n">
+      <c r="A72" t="n">
         <v>70</v>
       </c>
       <c r="B72" t="n">
@@ -1222,7 +1210,7 @@
       </c>
     </row>
     <row r="73">
-      <c r="A73" s="1" t="n">
+      <c r="A73" t="n">
         <v>71</v>
       </c>
       <c r="B73" t="n">
@@ -1233,7 +1221,7 @@
       </c>
     </row>
     <row r="74">
-      <c r="A74" s="1" t="n">
+      <c r="A74" t="n">
         <v>72</v>
       </c>
       <c r="B74" t="n">
@@ -1244,7 +1232,7 @@
       </c>
     </row>
     <row r="75">
-      <c r="A75" s="1" t="n">
+      <c r="A75" t="n">
         <v>73</v>
       </c>
       <c r="B75" t="n">
@@ -1255,7 +1243,7 @@
       </c>
     </row>
     <row r="76">
-      <c r="A76" s="1" t="n">
+      <c r="A76" t="n">
         <v>74</v>
       </c>
       <c r="B76" t="n">
@@ -1266,7 +1254,7 @@
       </c>
     </row>
     <row r="77">
-      <c r="A77" s="1" t="n">
+      <c r="A77" t="n">
         <v>75</v>
       </c>
       <c r="B77" t="n">
@@ -1277,7 +1265,7 @@
       </c>
     </row>
     <row r="78">
-      <c r="A78" s="1" t="n">
+      <c r="A78" t="n">
         <v>76</v>
       </c>
       <c r="B78" t="n">
@@ -1288,7 +1276,7 @@
       </c>
     </row>
     <row r="79">
-      <c r="A79" s="1" t="n">
+      <c r="A79" t="n">
         <v>77</v>
       </c>
       <c r="B79" t="n">
@@ -1299,7 +1287,7 @@
       </c>
     </row>
     <row r="80">
-      <c r="A80" s="1" t="n">
+      <c r="A80" t="n">
         <v>78</v>
       </c>
       <c r="B80" t="n">
@@ -1310,7 +1298,7 @@
       </c>
     </row>
     <row r="81">
-      <c r="A81" s="1" t="n">
+      <c r="A81" t="n">
         <v>79</v>
       </c>
       <c r="B81" t="n">
@@ -1321,7 +1309,7 @@
       </c>
     </row>
     <row r="82">
-      <c r="A82" s="1" t="n">
+      <c r="A82" t="n">
         <v>80</v>
       </c>
       <c r="B82" t="n">
@@ -1332,7 +1320,7 @@
       </c>
     </row>
     <row r="83">
-      <c r="A83" s="1" t="n">
+      <c r="A83" t="n">
         <v>81</v>
       </c>
       <c r="B83" t="n">
@@ -1343,7 +1331,7 @@
       </c>
     </row>
     <row r="84">
-      <c r="A84" s="1" t="n">
+      <c r="A84" t="n">
         <v>82</v>
       </c>
       <c r="B84" t="n">
@@ -1354,7 +1342,7 @@
       </c>
     </row>
     <row r="85">
-      <c r="A85" s="1" t="n">
+      <c r="A85" t="n">
         <v>83</v>
       </c>
       <c r="B85" t="n">
@@ -1365,7 +1353,7 @@
       </c>
     </row>
     <row r="86">
-      <c r="A86" s="1" t="n">
+      <c r="A86" t="n">
         <v>84</v>
       </c>
       <c r="B86" t="n">
@@ -1376,7 +1364,7 @@
       </c>
     </row>
     <row r="87">
-      <c r="A87" s="1" t="n">
+      <c r="A87" t="n">
         <v>85</v>
       </c>
       <c r="B87" t="n">
@@ -1387,7 +1375,7 @@
       </c>
     </row>
     <row r="88">
-      <c r="A88" s="1" t="n">
+      <c r="A88" t="n">
         <v>86</v>
       </c>
       <c r="B88" t="n">
@@ -1398,7 +1386,7 @@
       </c>
     </row>
     <row r="89">
-      <c r="A89" s="1" t="n">
+      <c r="A89" t="n">
         <v>87</v>
       </c>
       <c r="B89" t="n">
@@ -1409,7 +1397,7 @@
       </c>
     </row>
     <row r="90">
-      <c r="A90" s="1" t="n">
+      <c r="A90" t="n">
         <v>88</v>
       </c>
       <c r="B90" t="n">
@@ -1420,7 +1408,7 @@
       </c>
     </row>
     <row r="91">
-      <c r="A91" s="1" t="n">
+      <c r="A91" t="n">
         <v>89</v>
       </c>
       <c r="B91" t="n">
@@ -1431,7 +1419,7 @@
       </c>
     </row>
     <row r="92">
-      <c r="A92" s="1" t="n">
+      <c r="A92" t="n">
         <v>90</v>
       </c>
       <c r="B92" t="n">
@@ -1442,7 +1430,7 @@
       </c>
     </row>
     <row r="93">
-      <c r="A93" s="1" t="n">
+      <c r="A93" t="n">
         <v>91</v>
       </c>
       <c r="B93" t="n">
@@ -1453,7 +1441,7 @@
       </c>
     </row>
     <row r="94">
-      <c r="A94" s="1" t="n">
+      <c r="A94" t="n">
         <v>92</v>
       </c>
       <c r="B94" t="n">

</xml_diff>